<commit_message>
Monte Carlo simulation for the fuel tank filter project
</commit_message>
<xml_diff>
--- a/dataset/C2019-05 Fuel Tank Filter.xlsx
+++ b/dataset/C2019-05 Fuel Tank Filter.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1" documentId="11_97029EF239CC8C1758F89AC99BC57D4F5E1E0C12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91F2D576-4007-465F-A062-E65314A527C4}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13850" yWindow="120" windowWidth="24480" windowHeight="20760" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Schedule" sheetId="1" r:id="rId1"/>
@@ -33,8 +33,19 @@
     <sheet name="SPI, SPI(t), p-factor" sheetId="18" r:id="rId18"/>
     <sheet name="Corrective actions Overview" sheetId="19" r:id="rId19"/>
   </sheets>
-  <calcPr calcId="124519" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -3043,6 +3054,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>